<commit_message>
Update status: hipoteques 2026-06-21
</commit_message>
<xml_diff>
--- a/docs/hipoteques.xlsx
+++ b/docs/hipoteques.xlsx
@@ -1653,42 +1653,6 @@
           <t>202602</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>59531</v>
-      </c>
-      <c r="F2" t="n">
-        <v>58459</v>
-      </c>
-      <c r="J2" t="n">
-        <v>46661</v>
-      </c>
-      <c r="N2" t="n">
-        <v>458</v>
-      </c>
-      <c r="R2" t="n">
-        <v>11340</v>
-      </c>
-      <c r="V2" t="n">
-        <v>1072</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>11478708</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>11150811</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>8125195</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>408039</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>2617577</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>327897</v>
-      </c>
       <c r="AX2" t="n">
         <v>69425</v>
       </c>
@@ -1714,42 +1678,6 @@
           <t>202601</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>59349</v>
-      </c>
-      <c r="F3" t="n">
-        <v>58406</v>
-      </c>
-      <c r="J3" t="n">
-        <v>45563</v>
-      </c>
-      <c r="N3" t="n">
-        <v>507</v>
-      </c>
-      <c r="R3" t="n">
-        <v>12336</v>
-      </c>
-      <c r="V3" t="n">
-        <v>943</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>11181160</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>10983495</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>7895166</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>477874</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>2610455</v>
-      </c>
-      <c r="AT3" t="n">
-        <v>197665</v>
-      </c>
       <c r="AX3" t="n">
         <v>55864</v>
       </c>
@@ -1775,42 +1703,6 @@
           <t>202512</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>49384</v>
-      </c>
-      <c r="F4" t="n">
-        <v>48585</v>
-      </c>
-      <c r="J4" t="n">
-        <v>39330</v>
-      </c>
-      <c r="N4" t="n">
-        <v>404</v>
-      </c>
-      <c r="R4" t="n">
-        <v>8851</v>
-      </c>
-      <c r="V4" t="n">
-        <v>799</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>9949811</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>9782222</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>6665198</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>424379</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>2692645</v>
-      </c>
-      <c r="AT4" t="n">
-        <v>167589</v>
-      </c>
       <c r="AX4" t="n">
         <v>59062</v>
       </c>
@@ -1836,42 +1728,6 @@
           <t>202511</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>49271</v>
-      </c>
-      <c r="F5" t="n">
-        <v>48290</v>
-      </c>
-      <c r="J5" t="n">
-        <v>37841</v>
-      </c>
-      <c r="N5" t="n">
-        <v>487</v>
-      </c>
-      <c r="R5" t="n">
-        <v>9962</v>
-      </c>
-      <c r="V5" t="n">
-        <v>981</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>9878599</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>9608183</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>6528887</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>545099</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>2534197</v>
-      </c>
-      <c r="AT5" t="n">
-        <v>270416</v>
-      </c>
       <c r="AX5" t="n">
         <v>54979</v>
       </c>
@@ -1897,42 +1753,6 @@
           <t>202510</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>55762</v>
-      </c>
-      <c r="F6" t="n">
-        <v>54928</v>
-      </c>
-      <c r="J6" t="n">
-        <v>43319</v>
-      </c>
-      <c r="N6" t="n">
-        <v>368</v>
-      </c>
-      <c r="R6" t="n">
-        <v>11241</v>
-      </c>
-      <c r="V6" t="n">
-        <v>834</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>10695781</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>10510935</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>7397618</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>265620</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>2847697</v>
-      </c>
-      <c r="AT6" t="n">
-        <v>184846</v>
-      </c>
       <c r="AX6" t="n">
         <v>62184</v>
       </c>
@@ -1958,42 +1778,6 @@
           <t>202509</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>66960</v>
-      </c>
-      <c r="F7" t="n">
-        <v>65863</v>
-      </c>
-      <c r="J7" t="n">
-        <v>52198</v>
-      </c>
-      <c r="N7" t="n">
-        <v>367</v>
-      </c>
-      <c r="R7" t="n">
-        <v>13298</v>
-      </c>
-      <c r="V7" t="n">
-        <v>1097</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>12252940</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>11988179</v>
-      </c>
-      <c r="AH7" t="n">
-        <v>8721246</v>
-      </c>
-      <c r="AL7" t="n">
-        <v>443243</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>2823690</v>
-      </c>
-      <c r="AT7" t="n">
-        <v>264761</v>
-      </c>
       <c r="AX7" t="n">
         <v>67202</v>
       </c>
@@ -2019,42 +1803,6 @@
           <t>202508</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>59261</v>
-      </c>
-      <c r="F8" t="n">
-        <v>58227</v>
-      </c>
-      <c r="J8" t="n">
-        <v>46120</v>
-      </c>
-      <c r="N8" t="n">
-        <v>479</v>
-      </c>
-      <c r="R8" t="n">
-        <v>11628</v>
-      </c>
-      <c r="V8" t="n">
-        <v>1034</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>11566816</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>11360334</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>7914755</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>528921</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>2916658</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>206482</v>
-      </c>
       <c r="AX8" t="n">
         <v>52829</v>
       </c>
@@ -2080,42 +1828,6 @@
           <t>202507</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>43089</v>
-      </c>
-      <c r="F9" t="n">
-        <v>42407</v>
-      </c>
-      <c r="J9" t="n">
-        <v>33271</v>
-      </c>
-      <c r="N9" t="n">
-        <v>272</v>
-      </c>
-      <c r="R9" t="n">
-        <v>8864</v>
-      </c>
-      <c r="V9" t="n">
-        <v>682</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>8129264</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>7990659</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>5644431</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>370208</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>1976020</v>
-      </c>
-      <c r="AT9" t="n">
-        <v>138605</v>
-      </c>
       <c r="AX9" t="n">
         <v>40817</v>
       </c>
@@ -2141,42 +1853,6 @@
           <t>202506</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>57299</v>
-      </c>
-      <c r="F10" t="n">
-        <v>56431</v>
-      </c>
-      <c r="J10" t="n">
-        <v>45067</v>
-      </c>
-      <c r="N10" t="n">
-        <v>419</v>
-      </c>
-      <c r="R10" t="n">
-        <v>10945</v>
-      </c>
-      <c r="V10" t="n">
-        <v>868</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>10385897</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>10194623</v>
-      </c>
-      <c r="AH10" t="n">
-        <v>7359757</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>352831</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>2482035</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>191274</v>
-      </c>
       <c r="AX10" t="n">
         <v>58877</v>
       </c>
@@ -2202,42 +1878,6 @@
           <t>202505</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>53438</v>
-      </c>
-      <c r="F11" t="n">
-        <v>52654</v>
-      </c>
-      <c r="J11" t="n">
-        <v>41834</v>
-      </c>
-      <c r="N11" t="n">
-        <v>497</v>
-      </c>
-      <c r="R11" t="n">
-        <v>10323</v>
-      </c>
-      <c r="V11" t="n">
-        <v>784</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>9778252</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>9604368</v>
-      </c>
-      <c r="AH11" t="n">
-        <v>7043297</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>469554</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>2091517</v>
-      </c>
-      <c r="AT11" t="n">
-        <v>173884</v>
-      </c>
       <c r="AX11" t="n">
         <v>59150</v>
       </c>
@@ -2263,42 +1903,6 @@
           <t>202504</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>54744</v>
-      </c>
-      <c r="F12" t="n">
-        <v>53860</v>
-      </c>
-      <c r="J12" t="n">
-        <v>42274</v>
-      </c>
-      <c r="N12" t="n">
-        <v>382</v>
-      </c>
-      <c r="R12" t="n">
-        <v>11204</v>
-      </c>
-      <c r="V12" t="n">
-        <v>884</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>9367997</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>9168572</v>
-      </c>
-      <c r="AH12" t="n">
-        <v>6685742</v>
-      </c>
-      <c r="AL12" t="n">
-        <v>309641</v>
-      </c>
-      <c r="AP12" t="n">
-        <v>2173189</v>
-      </c>
-      <c r="AT12" t="n">
-        <v>199425</v>
-      </c>
       <c r="AX12" t="n">
         <v>58125</v>
       </c>
@@ -2323,42 +1927,6 @@
         <is>
           <t>202503</t>
         </is>
-      </c>
-      <c r="B13" t="n">
-        <v>50562</v>
-      </c>
-      <c r="F13" t="n">
-        <v>49869</v>
-      </c>
-      <c r="J13" t="n">
-        <v>39176</v>
-      </c>
-      <c r="N13" t="n">
-        <v>349</v>
-      </c>
-      <c r="R13" t="n">
-        <v>10344</v>
-      </c>
-      <c r="V13" t="n">
-        <v>693</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>8620259</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>8295254</v>
-      </c>
-      <c r="AH13" t="n">
-        <v>6106866</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>337654</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>1850734</v>
-      </c>
-      <c r="AT13" t="n">
-        <v>325005</v>
       </c>
       <c r="AX13" t="n">
         <v>55304</v>

</xml_diff>